<commit_message>
Updated CAN_grids_kan model - 2025-11-11 19:33
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CAN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A07B03B-F9EE-4952-855F-A3261CA809E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{381D7B45-173E-483B-8CE5-6D8E49B2ACBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29364,7 +29364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA8E3465-7C23-43A2-927F-82AD1F72E626}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC484AB-B0D3-4B25-BBE3-46CA4BB7B4D3}">
   <dimension ref="B9:H833"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -45610,7 +45610,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2702B8D5-FFE9-4125-B24E-64F37DF6938E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{868CA34F-E405-4AFB-98A7-B5C97A86D596}">
   <dimension ref="B9:L833"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN_grids_kan model - 2025-11-11 23:15
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CAN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{381D7B45-173E-483B-8CE5-6D8E49B2ACBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{75F2F641-E5A3-4C68-A204-A49E48E2EC59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29364,7 +29364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC484AB-B0D3-4B25-BBE3-46CA4BB7B4D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BE967C9-DA71-4557-9A07-3391E7CB221D}">
   <dimension ref="B9:H833"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -45610,7 +45610,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{868CA34F-E405-4AFB-98A7-B5C97A86D596}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9170B912-8FFE-454A-B3CE-FEB09F497336}">
   <dimension ref="B9:L833"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN_grids_kan model - 2025-11-11 23:36
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CAN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{75F2F641-E5A3-4C68-A204-A49E48E2EC59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F2BFF51-072D-4B34-BF1B-0ECC0DFA742B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29364,7 +29364,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BE967C9-DA71-4557-9A07-3391E7CB221D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB5F532-440B-4334-A6B0-5335BEDB6E52}">
   <dimension ref="B9:H833"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -45610,7 +45610,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9170B912-8FFE-454A-B3CE-FEB09F497336}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26701883-321E-49FB-A1DE-15109595879D}">
   <dimension ref="B9:L833"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>